<commit_message>
Update macroeconomic data file with new indicators and classifications
- Revised the existing Excel file to include updated macroeconomic indicators, enhancing the dataset for analysis.
- Ensured the file structure aligns with current documentation standards, maintaining clarity and usability for users.
</commit_message>
<xml_diff>
--- a/docs/指标确认表格/市场分析需求-数据采购确认清单v3.xlsx
+++ b/docs/指标确认表格/市场分析需求-数据采购确认清单v3.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13340" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="15240"/>
   </bookViews>
   <sheets>
     <sheet name="宏观数据" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="258">
   <si>
     <t>■ 1. 经济增长与景气</t>
   </si>
@@ -93,363 +93,360 @@
     <t>季频</t>
   </si>
   <si>
+    <t>近10年</t>
+  </si>
+  <si>
+    <t>YoY</t>
+  </si>
+  <si>
+    <t>经济总量主锚</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>1.2 景气度</t>
+  </si>
+  <si>
+    <t>PMI_MANU</t>
+  </si>
+  <si>
+    <t>EMM00121996</t>
+  </si>
+  <si>
+    <t>中国:PMI</t>
+  </si>
+  <si>
+    <t>月度</t>
+  </si>
+  <si>
+    <t>月频</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>景气主锚</t>
+  </si>
+  <si>
+    <t>PMI_SERV</t>
+  </si>
+  <si>
+    <t>EMM00122009</t>
+  </si>
+  <si>
+    <t>中国:非制造业PMI:商务活动</t>
+  </si>
+  <si>
+    <t>服务景气</t>
+  </si>
+  <si>
+    <t>1.3 工业与生产</t>
+  </si>
+  <si>
+    <t>INDUSTRY_YOY</t>
+  </si>
+  <si>
+    <t>EMM00008445</t>
+  </si>
+  <si>
+    <t>中国:工业增加值:同比</t>
+  </si>
+  <si>
+    <t>生产侧增长</t>
+  </si>
+  <si>
+    <t>■ 2. 通胀与价格</t>
+  </si>
+  <si>
+    <t>CPI_YOY</t>
+  </si>
+  <si>
+    <t>EMM00072301</t>
+  </si>
+  <si>
+    <t>中国:CPI:同比</t>
+  </si>
+  <si>
+    <t>居民通胀主锚</t>
+  </si>
+  <si>
+    <t>PPI_YOY</t>
+  </si>
+  <si>
+    <t>EMM00073348</t>
+  </si>
+  <si>
+    <t>中国:PPI:全部工业品:同比</t>
+  </si>
+  <si>
+    <t>工业通胀 / 价格传导</t>
+  </si>
+  <si>
+    <t>■ 3. 消费与居民部门</t>
+  </si>
+  <si>
+    <t>RETAIL_SALES_YOY</t>
+  </si>
+  <si>
+    <t>EMM00063225</t>
+  </si>
+  <si>
+    <t>中国:社会消费品零售总额:累计同比</t>
+  </si>
+  <si>
+    <t>消费结果指标</t>
+  </si>
+  <si>
+    <t>URBAN_DISPOSABLE_INCOME_CUM_YOY</t>
+  </si>
+  <si>
+    <t>EMM00597048</t>
+  </si>
+  <si>
+    <t>中国:城镇居民人均可支配收入:累计同比</t>
+  </si>
+  <si>
+    <t>累计YoY</t>
+  </si>
+  <si>
+    <t>居民收入支撑</t>
+  </si>
+  <si>
+    <t>CONSUMER_CONFIDENCE</t>
+  </si>
+  <si>
+    <t>EMM00122031</t>
+  </si>
+  <si>
+    <t>中国:消费者信心指数</t>
+  </si>
+  <si>
+    <t>NBS / Wind / Choice</t>
+  </si>
+  <si>
+    <t>消费预期主锚</t>
+  </si>
+  <si>
+    <t>■ 4. 投资与房地产</t>
+  </si>
+  <si>
+    <t>4.1 投资</t>
+  </si>
+  <si>
+    <t>INFRA_INVEST_CUM_YOY</t>
+  </si>
+  <si>
+    <t>EMM00597116</t>
+  </si>
+  <si>
+    <t>中国:城镇固定资产投资完成额:基础设施(不含电力):累计同比</t>
+  </si>
+  <si>
+    <t>投资三分法之一</t>
+  </si>
+  <si>
+    <t>MANUFACTURING_INVEST_CUM_YOY</t>
+  </si>
+  <si>
+    <t>EMM00027220</t>
+  </si>
+  <si>
+    <t>中国:固定资产投资完成额:制造业:累计同比</t>
+  </si>
+  <si>
+    <t>REAL_ESTATE_INVEST_CUM_YOY</t>
+  </si>
+  <si>
+    <t>EMI00120220</t>
+  </si>
+  <si>
+    <t>中国:房地产开发投资完成额:累计同比</t>
+  </si>
+  <si>
+    <t>4.2 房地产</t>
+  </si>
+  <si>
+    <t>RESID_HOUSE_SALES_CUMULATIVE_YOY</t>
+  </si>
+  <si>
+    <t>EMM00877640</t>
+  </si>
+  <si>
+    <t>商品房销售额:住宅:累计同比</t>
+  </si>
+  <si>
+    <t>地产需求验证</t>
+  </si>
+  <si>
+    <t>PROPERTY_SALES_AREA_30CITIES_ROLLING12M_YOY</t>
+  </si>
+  <si>
+    <t>EMI01778652</t>
+  </si>
+  <si>
+    <t>中国:30大中城市:商品房成交面积:滚动12个月同比</t>
+  </si>
+  <si>
+    <t>Wind / Choice</t>
+  </si>
+  <si>
+    <t>滚动12M同比</t>
+  </si>
+  <si>
+    <t>地产高频成交验证</t>
+  </si>
+  <si>
+    <t>HOUSE_PRICE_70CITY_SECONDHAND_YOY</t>
+  </si>
+  <si>
+    <t>EMI01736192</t>
+  </si>
+  <si>
+    <t>中国:70大中城市二手住宅价格指数:当月同比</t>
+  </si>
+  <si>
+    <t>房价趋势主锚</t>
+  </si>
+  <si>
+    <t>■ 5. 外需、贸易与汇率</t>
+  </si>
+  <si>
+    <t>EXPORT_CUMULATIVE_YOY</t>
+  </si>
+  <si>
+    <t>EMM00183416</t>
+  </si>
+  <si>
+    <t>中国:出口金额:累计同比</t>
+  </si>
+  <si>
+    <t>海关总署</t>
+  </si>
+  <si>
+    <t>出口结果指标</t>
+  </si>
+  <si>
+    <t>IMPORT_CUMULATIVE_YOY</t>
+  </si>
+  <si>
+    <t>EMM00042521</t>
+  </si>
+  <si>
+    <t>中国:进口金额:累计同比</t>
+  </si>
+  <si>
+    <t>进口结果指标</t>
+  </si>
+  <si>
+    <t>PMI_NEW_EXPORT_ORDERS</t>
+  </si>
+  <si>
+    <t>EMM00121999</t>
+  </si>
+  <si>
+    <t>中国:PMI:新出口订单</t>
+  </si>
+  <si>
+    <t>出口前瞻指标</t>
+  </si>
+  <si>
+    <t>FX_CNY_MID</t>
+  </si>
+  <si>
+    <t>EMM00058124</t>
+  </si>
+  <si>
+    <t>中间价:美元兑人民币</t>
+  </si>
+  <si>
+    <t>PBOC</t>
+  </si>
+  <si>
+    <t>日度</t>
+  </si>
+  <si>
+    <t>日频</t>
+  </si>
+  <si>
+    <t>汇率与外部冲击传导</t>
+  </si>
+  <si>
+    <t>■ 6. 货币、信用与利率</t>
+  </si>
+  <si>
+    <t>6.1 货币</t>
+  </si>
+  <si>
+    <t>M2_YOY</t>
+  </si>
+  <si>
+    <t>EMM00087086</t>
+  </si>
+  <si>
+    <t>中国:M2:同比</t>
+  </si>
+  <si>
+    <t>流动性主锚</t>
+  </si>
+  <si>
+    <t>M1_YOY</t>
+  </si>
+  <si>
+    <t>EMM00087084</t>
+  </si>
+  <si>
+    <t>中国:M1:同比</t>
+  </si>
+  <si>
+    <t>货币活性主锚</t>
+  </si>
+  <si>
+    <t>DR007</t>
+  </si>
+  <si>
+    <t>E1300004</t>
+  </si>
+  <si>
+    <t>CFETS</t>
+  </si>
+  <si>
+    <t>日频（保留原始+输出月均）</t>
+  </si>
+  <si>
+    <t>资金价格锚</t>
+  </si>
+  <si>
+    <t>6.2 信用</t>
+  </si>
+  <si>
+    <t>TSF_STOCK_YOY</t>
+  </si>
+  <si>
+    <t>EMM00634721</t>
+  </si>
+  <si>
+    <t>中国:社会融资规模存量:同比</t>
+  </si>
+  <si>
+    <t>信用周期主锚</t>
+  </si>
+  <si>
+    <t>AA_CREDIT_YIELD_3Y</t>
+  </si>
+  <si>
+    <t>E1000469</t>
+  </si>
+  <si>
+    <t>AA级信用债收益率（3年）</t>
+  </si>
+  <si>
+    <t>中债 / Wind / Choice</t>
+  </si>
+  <si>
     <t>近20年</t>
   </si>
   <si>
-    <t>YoY</t>
-  </si>
-  <si>
-    <t>经济总量主锚</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>1.2 景气度</t>
-  </si>
-  <si>
-    <t>PMI_MANU</t>
-  </si>
-  <si>
-    <t>EMM00121996</t>
-  </si>
-  <si>
-    <t>中国:PMI</t>
-  </si>
-  <si>
-    <t>月度</t>
-  </si>
-  <si>
-    <t>月频</t>
-  </si>
-  <si>
-    <t>Level</t>
-  </si>
-  <si>
-    <t>景气主锚</t>
-  </si>
-  <si>
-    <t>PMI_SERV</t>
-  </si>
-  <si>
-    <t>EMM00122009</t>
-  </si>
-  <si>
-    <t>中国:非制造业PMI:商务活动</t>
-  </si>
-  <si>
-    <t>服务景气</t>
-  </si>
-  <si>
-    <t>1.3 工业与生产</t>
-  </si>
-  <si>
-    <t>INDUSTRY_YOY</t>
-  </si>
-  <si>
-    <t>EMM00008445</t>
-  </si>
-  <si>
-    <t>中国:工业增加值:同比</t>
-  </si>
-  <si>
-    <t>生产侧增长</t>
-  </si>
-  <si>
-    <t>■ 2. 通胀与价格</t>
-  </si>
-  <si>
-    <t>CPI_YOY</t>
-  </si>
-  <si>
-    <t>EMM00072301</t>
-  </si>
-  <si>
-    <t>中国:CPI:同比</t>
-  </si>
-  <si>
-    <t>居民通胀主锚</t>
-  </si>
-  <si>
-    <t>PPI_YOY</t>
-  </si>
-  <si>
-    <t>EMM00073348</t>
-  </si>
-  <si>
-    <t>中国:PPI:全部工业品:同比</t>
-  </si>
-  <si>
-    <t>工业通胀 / 价格传导</t>
-  </si>
-  <si>
-    <t>■ 3. 消费与居民部门</t>
-  </si>
-  <si>
-    <t>RETAIL_SALES_YOY</t>
-  </si>
-  <si>
-    <t>EMM00063225</t>
-  </si>
-  <si>
-    <t>中国:社会消费品零售总额:累计同比</t>
-  </si>
-  <si>
-    <t>近10年</t>
-  </si>
-  <si>
-    <t>消费结果指标</t>
-  </si>
-  <si>
-    <t>URBAN_DISPOSABLE_INCOME_CUM_YOY</t>
-  </si>
-  <si>
-    <t>EMM00597048</t>
-  </si>
-  <si>
-    <t>中国:城镇居民人均可支配收入:累计同比</t>
-  </si>
-  <si>
-    <t>累计YoY</t>
-  </si>
-  <si>
-    <t>居民收入支撑</t>
-  </si>
-  <si>
-    <t>CONSUMER_CONFIDENCE</t>
-  </si>
-  <si>
-    <t>EMM00122031</t>
-  </si>
-  <si>
-    <t>中国:消费者信心指数</t>
-  </si>
-  <si>
-    <t>NBS / Wind / Choice</t>
-  </si>
-  <si>
-    <t>消费预期主锚</t>
-  </si>
-  <si>
-    <t>■ 4. 投资与房地产</t>
-  </si>
-  <si>
-    <t>4.1 投资</t>
-  </si>
-  <si>
-    <t>INFRA_INVEST_CUM_YOY</t>
-  </si>
-  <si>
-    <t>EMM00597116</t>
-  </si>
-  <si>
-    <t>中国:城镇固定资产投资完成额:基础设施(不含电力):累计同比</t>
-  </si>
-  <si>
-    <t>投资三分法之一</t>
-  </si>
-  <si>
-    <t>MANUFACTURING_INVEST_CUM_YOY</t>
-  </si>
-  <si>
-    <t>EMM00027220</t>
-  </si>
-  <si>
-    <t>中国:固定资产投资完成额:制造业:累计同比</t>
-  </si>
-  <si>
-    <t>REAL_ESTATE_INVEST_CUM_YOY</t>
-  </si>
-  <si>
-    <t>EMI00120220</t>
-  </si>
-  <si>
-    <t>中国:房地产开发投资完成额:累计同比</t>
-  </si>
-  <si>
-    <t>4.2 房地产</t>
-  </si>
-  <si>
-    <t>RESID_HOUSE_SALES_CUMULATIVE_YOY</t>
-  </si>
-  <si>
-    <t>EMM00877640</t>
-  </si>
-  <si>
-    <t>商品房销售额:住宅:累计同比</t>
-  </si>
-  <si>
-    <t>地产需求验证</t>
-  </si>
-  <si>
-    <t>PROPERTY_SALES_AREA_30CITIES_ROLLING12M_YOY</t>
-  </si>
-  <si>
-    <t>EMI01778652</t>
-  </si>
-  <si>
-    <t>中国:30大中城市:商品房成交面积:滚动12个月同比</t>
-  </si>
-  <si>
-    <t>Wind / Choice</t>
-  </si>
-  <si>
-    <t>近10-15年</t>
-  </si>
-  <si>
-    <t>滚动12M同比</t>
-  </si>
-  <si>
-    <t>地产高频成交验证</t>
-  </si>
-  <si>
-    <t>HOUSE_PRICE_70CITY_SECONDHAND_YOY</t>
-  </si>
-  <si>
-    <t>EMI01736192</t>
-  </si>
-  <si>
-    <t>中国:70大中城市二手住宅价格指数:当月同比</t>
-  </si>
-  <si>
-    <t>房价趋势主锚</t>
-  </si>
-  <si>
-    <t>■ 5. 外需、贸易与汇率</t>
-  </si>
-  <si>
-    <t>EXPORT_CUMULATIVE_YOY</t>
-  </si>
-  <si>
-    <t>EMM00183416</t>
-  </si>
-  <si>
-    <t>中国:出口金额:累计同比</t>
-  </si>
-  <si>
-    <t>海关总署</t>
-  </si>
-  <si>
-    <t>出口结果指标</t>
-  </si>
-  <si>
-    <t>IMPORT_CUMULATIVE_YOY</t>
-  </si>
-  <si>
-    <t>EMM00042521</t>
-  </si>
-  <si>
-    <t>中国:进口金额:累计同比</t>
-  </si>
-  <si>
-    <t>进口结果指标</t>
-  </si>
-  <si>
-    <t>PMI_NEW_EXPORT_ORDERS</t>
-  </si>
-  <si>
-    <t>EMM00121999</t>
-  </si>
-  <si>
-    <t>中国:PMI:新出口订单</t>
-  </si>
-  <si>
-    <t>出口前瞻指标</t>
-  </si>
-  <si>
-    <t>FX_CNY_MID</t>
-  </si>
-  <si>
-    <t>EMM00058124</t>
-  </si>
-  <si>
-    <t>中间价:美元兑人民币</t>
-  </si>
-  <si>
-    <t>PBOC</t>
-  </si>
-  <si>
-    <t>日度</t>
-  </si>
-  <si>
-    <t>日频</t>
-  </si>
-  <si>
-    <t>汇率与外部冲击传导</t>
-  </si>
-  <si>
-    <t>■ 6. 货币、信用与利率</t>
-  </si>
-  <si>
-    <t>6.1 货币</t>
-  </si>
-  <si>
-    <t>M2_YOY</t>
-  </si>
-  <si>
-    <t>EMM00087086</t>
-  </si>
-  <si>
-    <t>中国:M2:同比</t>
-  </si>
-  <si>
-    <t>流动性主锚</t>
-  </si>
-  <si>
-    <t>M1_YOY</t>
-  </si>
-  <si>
-    <t>EMM00087084</t>
-  </si>
-  <si>
-    <t>中国:M1:同比</t>
-  </si>
-  <si>
-    <t>货币活性主锚</t>
-  </si>
-  <si>
-    <t>DR007</t>
-  </si>
-  <si>
-    <t>E1300004</t>
-  </si>
-  <si>
-    <t>CFETS</t>
-  </si>
-  <si>
-    <t>日频（保留原始+输出月均）</t>
-  </si>
-  <si>
-    <t>资金价格锚</t>
-  </si>
-  <si>
-    <t>6.2 信用</t>
-  </si>
-  <si>
-    <t>TSF_STOCK_YOY</t>
-  </si>
-  <si>
-    <t>EMM00634721</t>
-  </si>
-  <si>
-    <t>中国:社会融资规模存量:同比</t>
-  </si>
-  <si>
-    <t>信用周期主锚</t>
-  </si>
-  <si>
-    <t>AA_CREDIT_YIELD_3Y</t>
-  </si>
-  <si>
-    <t>E1000469</t>
-  </si>
-  <si>
-    <t>AA级信用债收益率（3年）</t>
-  </si>
-  <si>
-    <t>中债 / Wind / Choice</t>
-  </si>
-  <si>
     <t>信用风险主锚</t>
   </si>
   <si>
@@ -465,9 +462,6 @@
     <t>中债国债到期收益率:1年</t>
   </si>
   <si>
-    <t>近15-20年</t>
-  </si>
-  <si>
     <t>建模无风险利率</t>
   </si>
   <si>
@@ -504,9 +498,6 @@
     <t>贷款市场报价利率(LPR):1年</t>
   </si>
   <si>
-    <t>2019-08起</t>
-  </si>
-  <si>
     <t>价格型政策工具 / 金融条件变量</t>
   </si>
   <si>
@@ -522,9 +513,6 @@
     <t>PBOC / Choice</t>
   </si>
   <si>
-    <t>1999年至今</t>
-  </si>
-  <si>
     <t>数量型政策工具 / 流动性约束变量</t>
   </si>
   <si>
@@ -618,9 +606,6 @@
     <t>ICE / Wind / Choice</t>
   </si>
   <si>
-    <t>2013-06起</t>
-  </si>
-  <si>
     <t>全球通胀 / 地缘风险</t>
   </si>
   <si>
@@ -636,9 +621,6 @@
     <t>COMEX / Choice</t>
   </si>
   <si>
-    <t>1986-07起</t>
-  </si>
-  <si>
     <t>避险与另类资产驱动</t>
   </si>
   <si>
@@ -657,7 +639,19 @@
     <t>全球风险偏好代理</t>
   </si>
   <si>
-    <t>■ 9. 大类资产建模数据（额外建模指标）</t>
+    <r>
+      <t xml:space="preserve">■ 9. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF1F4E79"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>大类资产建模数据（额外建模指标）</t>
+    </r>
   </si>
   <si>
     <t>MMF_7D_YIELD_M</t>
@@ -672,9 +666,6 @@
     <t>Choice / 基金业协会 / Wind</t>
   </si>
   <si>
-    <t>2004-01至今</t>
-  </si>
-  <si>
     <t>方案A现金主腿</t>
   </si>
   <si>
@@ -687,9 +678,6 @@
     <t>中债新综合财富指数（固收类）</t>
   </si>
   <si>
-    <t>按可得最长</t>
-  </si>
-  <si>
     <t>方案A固收主腿 / 固收回测基准</t>
   </si>
   <si>
@@ -717,9 +705,6 @@
     <t>沪深300指数（股票类）</t>
   </si>
   <si>
-    <t>2005年至今</t>
-  </si>
-  <si>
     <t>方案B股票主腿</t>
   </si>
   <si>
@@ -748,6 +733,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF1F4E79"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">■ </t>
     </r>
     <r>
@@ -826,6 +818,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF1F4E79"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">■  </t>
     </r>
     <r>
@@ -903,11 +902,11 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体-简"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1433,19 +1432,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1454,7 +1453,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1604,11 +1603,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1974,7 +1973,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:12">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
@@ -1990,7 +1989,7 @@
       <c r="L1" s="3"/>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:12">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
@@ -2082,7 +2081,7 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:12">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="2"/>
@@ -2192,7 +2191,7 @@
       <c r="F8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H8" s="8" t="s">
@@ -2212,7 +2211,7 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:12">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="2"/>
@@ -2304,7 +2303,7 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:12">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B13" s="2"/>
@@ -2414,7 +2413,7 @@
       <c r="F16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H16" s="8" t="s">
@@ -2434,7 +2433,7 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:12">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B18" s="2"/>
@@ -2507,13 +2506,13 @@
         <v>29</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>21</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>23</v>
@@ -2527,13 +2526,13 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:12">
       <c r="A21" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>58</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>17</v>
@@ -2544,14 +2543,14 @@
       <c r="F21" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I21" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>60</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>23</v>
@@ -2565,16 +2564,16 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:12">
       <c r="A22" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>28</v>
@@ -2583,27 +2582,27 @@
         <v>29</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I22" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:12">
+      <c r="A24" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L22" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1" spans="1:12">
-      <c r="A24" s="11" t="s">
-        <v>66</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -2618,8 +2617,8 @@
       <c r="L24" s="3"/>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:12">
-      <c r="A25" s="12" t="s">
-        <v>67</v>
+      <c r="A25" s="11" t="s">
+        <v>66</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -2673,13 +2672,13 @@
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:12">
       <c r="A27" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>17</v>
@@ -2691,13 +2690,13 @@
         <v>29</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>23</v>
@@ -2711,13 +2710,13 @@
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:12">
       <c r="A28" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="C28" s="9" t="s">
         <v>73</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>17</v>
@@ -2729,13 +2728,13 @@
         <v>29</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>23</v>
@@ -2749,13 +2748,13 @@
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:12">
       <c r="A29" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>17</v>
@@ -2767,13 +2766,13 @@
         <v>29</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>23</v>
@@ -2786,8 +2785,8 @@
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:12">
-      <c r="A30" s="12" t="s">
-        <v>78</v>
+      <c r="A30" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -2841,13 +2840,13 @@
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:12">
       <c r="A32" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>17</v>
@@ -2859,13 +2858,13 @@
         <v>29</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>23</v>
@@ -2879,16 +2878,16 @@
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:12">
       <c r="A33" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="D33" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>86</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>28</v>
@@ -2896,14 +2895,14 @@
       <c r="F33" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="I33" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I33" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="J33" s="7" t="s">
         <v>23</v>
@@ -2917,16 +2916,16 @@
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:12">
       <c r="A34" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>92</v>
-      </c>
       <c r="D34" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>28</v>
@@ -2935,13 +2934,13 @@
         <v>29</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="H34" s="5" t="s">
         <v>21</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>23</v>
@@ -2954,8 +2953,8 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="1:12">
-      <c r="A36" s="11" t="s">
-        <v>94</v>
+      <c r="A36" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -3009,16 +3008,16 @@
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:12">
       <c r="A38" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="D38" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>28</v>
@@ -3027,13 +3026,13 @@
         <v>29</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J38" s="7" t="s">
         <v>23</v>
@@ -3047,16 +3046,16 @@
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:12">
       <c r="A39" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>102</v>
-      </c>
       <c r="D39" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E39" s="8" t="s">
         <v>28</v>
@@ -3065,13 +3064,13 @@
         <v>29</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J39" s="7" t="s">
         <v>23</v>
@@ -3085,13 +3084,13 @@
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:12">
       <c r="A40" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>106</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>17</v>
@@ -3103,13 +3102,13 @@
         <v>29</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="H40" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J40" s="7" t="s">
         <v>23</v>
@@ -3123,31 +3122,31 @@
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:12">
       <c r="A41" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="D41" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="E41" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="F41" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E41" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H41" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J41" s="7" t="s">
         <v>23</v>
@@ -3160,8 +3159,8 @@
       </c>
     </row>
     <row r="43" ht="18" customHeight="1" spans="1:12">
-      <c r="A43" s="11" t="s">
-        <v>115</v>
+      <c r="A43" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -3176,8 +3175,8 @@
       <c r="L43" s="3"/>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:12">
-      <c r="A44" s="12" t="s">
-        <v>116</v>
+      <c r="A44" s="11" t="s">
+        <v>114</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3231,16 +3230,16 @@
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:12">
       <c r="A46" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B46" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>119</v>
-      </c>
       <c r="D46" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>28</v>
@@ -3255,7 +3254,7 @@
         <v>21</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J46" s="7" t="s">
         <v>23</v>
@@ -3269,16 +3268,16 @@
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:12">
       <c r="A47" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="B47" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>123</v>
-      </c>
       <c r="D47" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>28</v>
@@ -3286,14 +3285,14 @@
       <c r="F47" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G47" s="8" t="s">
+      <c r="G47" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H47" s="8" t="s">
         <v>21</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J47" s="7" t="s">
         <v>23</v>
@@ -3307,22 +3306,22 @@
     </row>
     <row r="48" ht="15" customHeight="1" spans="1:12">
       <c r="A48" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="E48" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F48" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>20</v>
@@ -3331,7 +3330,7 @@
         <v>30</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J48" s="7" t="s">
         <v>23</v>
@@ -3344,8 +3343,8 @@
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:12">
-      <c r="A49" s="12" t="s">
-        <v>130</v>
+      <c r="A49" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -3399,16 +3398,16 @@
     </row>
     <row r="51" ht="15" customHeight="1" spans="1:12">
       <c r="A51" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="D51" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>28</v>
@@ -3423,7 +3422,7 @@
         <v>21</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J51" s="7" t="s">
         <v>23</v>
@@ -3437,45 +3436,45 @@
     </row>
     <row r="52" ht="15" customHeight="1" spans="1:12">
       <c r="A52" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C52" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="D52" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="E52" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="G52" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F52" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="H52" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I52" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="J52" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K52" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="L52" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1" spans="1:12">
+      <c r="A53" s="11" t="s">
         <v>139</v>
-      </c>
-      <c r="J52" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="K52" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L52" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="53" ht="16" customHeight="1" spans="1:12">
-      <c r="A53" s="12" t="s">
-        <v>140</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -3529,31 +3528,31 @@
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:12">
       <c r="A55" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B55" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="C55" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C55" s="6" t="s">
-        <v>143</v>
-      </c>
       <c r="D55" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>144</v>
+        <v>111</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="H55" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J55" s="7" t="s">
         <v>23</v>
@@ -3567,31 +3566,31 @@
     </row>
     <row r="56" ht="15" customHeight="1" spans="1:12">
       <c r="A56" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B56" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>148</v>
-      </c>
       <c r="D56" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H56" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J56" s="7" t="s">
         <v>23</v>
@@ -3605,31 +3604,31 @@
     </row>
     <row r="57" ht="15" customHeight="1" spans="1:12">
       <c r="A57" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C57" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B57" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>152</v>
-      </c>
       <c r="D57" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>87</v>
+        <v>111</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="H57" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J57" s="7" t="s">
         <v>23</v>
@@ -3643,16 +3642,16 @@
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:12">
       <c r="A58" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="B58" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>156</v>
-      </c>
       <c r="D58" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E58" s="8" t="s">
         <v>28</v>
@@ -3660,14 +3659,14 @@
       <c r="F58" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G58" s="8" t="s">
-        <v>157</v>
+      <c r="G58" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="H58" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I58" s="9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="J58" s="7" t="s">
         <v>23</v>
@@ -3681,16 +3680,16 @@
     </row>
     <row r="59" ht="15" customHeight="1" spans="1:12">
       <c r="A59" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="E59" s="5" t="s">
         <v>28</v>
@@ -3699,13 +3698,13 @@
         <v>29</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>163</v>
+        <v>20</v>
       </c>
       <c r="H59" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="J59" s="7" t="s">
         <v>23</v>
@@ -3718,8 +3717,8 @@
       </c>
     </row>
     <row r="61" ht="18" customHeight="1" spans="1:12">
-      <c r="A61" s="11" t="s">
-        <v>165</v>
+      <c r="A61" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -3734,8 +3733,8 @@
       <c r="L61" s="3"/>
     </row>
     <row r="62" ht="16" customHeight="1" spans="1:12">
-      <c r="A62" s="12" t="s">
-        <v>166</v>
+      <c r="A62" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -3789,13 +3788,13 @@
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:12">
       <c r="A64" s="6" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>17</v>
@@ -3807,13 +3806,13 @@
         <v>29</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="H64" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="J64" s="7" t="s">
         <v>23</v>
@@ -3826,8 +3825,8 @@
       </c>
     </row>
     <row r="65" ht="16" customHeight="1" spans="1:12">
-      <c r="A65" s="12" t="s">
-        <v>171</v>
+      <c r="A65" s="11" t="s">
+        <v>167</v>
       </c>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -3881,16 +3880,16 @@
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:12">
       <c r="A67" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>28</v>
@@ -3902,10 +3901,10 @@
         <v>20</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="J67" s="7" t="s">
         <v>23</v>
@@ -3919,16 +3918,16 @@
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:12">
       <c r="A68" s="9" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>28</v>
@@ -3936,14 +3935,14 @@
       <c r="F68" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G68" s="8" t="s">
-        <v>87</v>
+      <c r="G68" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J68" s="7" t="s">
         <v>23</v>
@@ -3957,31 +3956,31 @@
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:12">
       <c r="A69" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="F69" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C69" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>188</v>
-      </c>
       <c r="G69" s="5" t="s">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="H69" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="J69" s="7" t="s">
         <v>23</v>
@@ -3994,8 +3993,8 @@
       </c>
     </row>
     <row r="71" ht="18" customHeight="1" spans="1:12">
-      <c r="A71" s="11" t="s">
-        <v>190</v>
+      <c r="A71" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -4049,31 +4048,31 @@
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:12">
       <c r="A73" s="6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>195</v>
+        <v>20</v>
       </c>
       <c r="H73" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="J73" s="7" t="s">
         <v>23</v>
@@ -4087,31 +4086,31 @@
     </row>
     <row r="74" ht="15" customHeight="1" spans="1:12">
       <c r="A74" s="9" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G74" s="8" t="s">
-        <v>201</v>
+        <v>111</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="H74" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I74" s="9" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J74" s="7" t="s">
         <v>23</v>
@@ -4125,22 +4124,22 @@
     </row>
     <row r="75" ht="15" customHeight="1" spans="1:12">
       <c r="A75" s="6" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G75" s="5" t="s">
         <v>20</v>
@@ -4149,7 +4148,7 @@
         <v>30</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="J75" s="7" t="s">
         <v>23</v>
@@ -4162,8 +4161,8 @@
       </c>
     </row>
     <row r="77" ht="18" customHeight="1" spans="1:12">
-      <c r="A77" s="11" t="s">
-        <v>208</v>
+      <c r="A77" s="1" t="s">
+        <v>202</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4196,7 +4195,7 @@
       <c r="F78" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G78" s="4" t="s">
+      <c r="G78" s="12" t="s">
         <v>8</v>
       </c>
       <c r="H78" s="4" t="s">
@@ -4217,16 +4216,16 @@
     </row>
     <row r="79" ht="15" customHeight="1" spans="1:12">
       <c r="A79" s="6" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>28</v>
@@ -4235,13 +4234,13 @@
         <v>29</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>213</v>
+        <v>137</v>
       </c>
       <c r="H79" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="J79" s="7" t="s">
         <v>23</v>
@@ -4255,16 +4254,16 @@
     </row>
     <row r="80" ht="15" customHeight="1" spans="1:12">
       <c r="A80" s="9" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>28</v>
@@ -4272,14 +4271,14 @@
       <c r="F80" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G80" s="8" t="s">
-        <v>218</v>
+      <c r="G80" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="H80" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I80" s="9" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="J80" s="7" t="s">
         <v>23</v>
@@ -4293,31 +4292,31 @@
     </row>
     <row r="81" ht="15" customHeight="1" spans="1:12">
       <c r="A81" s="6" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>218</v>
+        <v>137</v>
       </c>
       <c r="H81" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="J81" s="7" t="s">
         <v>23</v>
@@ -4331,31 +4330,31 @@
     </row>
     <row r="82" ht="15" customHeight="1" spans="1:12">
       <c r="A82" s="9" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F82" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G82" s="8" t="s">
-        <v>228</v>
+        <v>111</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="H82" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I82" s="9" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="J82" s="7" t="s">
         <v>23</v>
@@ -4369,31 +4368,31 @@
     </row>
     <row r="83" ht="15" customHeight="1" spans="1:12">
       <c r="A83" s="6" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>20</v>
+        <v>137</v>
       </c>
       <c r="H83" s="5" t="s">
         <v>30</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="J83" s="7" t="s">
         <v>23</v>
@@ -4407,31 +4406,31 @@
     </row>
     <row r="84" ht="15" customHeight="1" spans="1:12">
       <c r="A84" s="9" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G84" s="8" t="s">
-        <v>20</v>
+        <v>137</v>
       </c>
       <c r="H84" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I84" s="9" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="J84" s="7" t="s">
         <v>23</v>
@@ -4489,7 +4488,7 @@
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4504,16 +4503,16 @@
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:11">
       <c r="A2" s="4" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>6</v>
@@ -4539,28 +4538,28 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:11">
       <c r="A3" s="5" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>23</v>
@@ -4574,28 +4573,28 @@
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:11">
       <c r="A4" s="8" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>23</v>
@@ -4609,28 +4608,28 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:11">
       <c r="A5" s="5" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>246</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>255</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>23</v>
@@ -4644,28 +4643,28 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:11">
       <c r="A6" s="8" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>23</v>
@@ -4679,7 +4678,7 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:11">
       <c r="A8" s="1" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -4726,25 +4725,25 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:11">
       <c r="A10" s="5" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>23</v>

</xml_diff>